<commit_message>
tested and finished implementing the HoF
</commit_message>
<xml_diff>
--- a/apps_nicolo/LogicCircuits_4s_5r_MAK_REINFORCE/LogicCircuits_5s_10r_MAK_REINFORCE.xlsx
+++ b/apps_nicolo/LogicCircuits_4s_5r_MAK_REINFORCE/LogicCircuits_5s_10r_MAK_REINFORCE.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$Y$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$Y$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y42"/>
+  <dimension ref="A1:Y49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
@@ -4173,8 +4173,589 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-12-04 16:48:14</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/dfe4086034af44ea8bcbe7d1988bbbfc</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H43" t="n">
+        <v>300</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>5</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L43" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M43" t="n">
+        <v>128</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>30</v>
+      </c>
+      <c r="R43" t="n">
+        <v>100</v>
+      </c>
+      <c r="S43" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T43" t="n">
+        <v>1</v>
+      </c>
+      <c r="U43" t="n">
+        <v>8</v>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-12-04 16:52:04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/8fed03a4518948508f74b3ff2208dcfa</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H44" t="n">
+        <v>300</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>5</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L44" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M44" t="n">
+        <v>128</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P44" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>30</v>
+      </c>
+      <c r="R44" t="n">
+        <v>100</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T44" t="n">
+        <v>1</v>
+      </c>
+      <c r="U44" t="n">
+        <v>8</v>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-12-04 16:58:37</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/a1b09948568a490aa61916627cfa1edb</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H45" t="n">
+        <v>300</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>5</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L45" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M45" t="n">
+        <v>128</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>30</v>
+      </c>
+      <c r="R45" t="n">
+        <v>100</v>
+      </c>
+      <c r="S45" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T45" t="n">
+        <v>1</v>
+      </c>
+      <c r="U45" t="n">
+        <v>8</v>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-12-04 17:04:02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/5c74df0dbc674f7ea8fa49ff0d68eee5</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H46" t="n">
+        <v>300</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>5</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L46" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M46" t="n">
+        <v>128</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>30</v>
+      </c>
+      <c r="R46" t="n">
+        <v>100</v>
+      </c>
+      <c r="S46" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T46" t="n">
+        <v>1</v>
+      </c>
+      <c r="U46" t="n">
+        <v>8</v>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-12-04 17:12:10</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/c64c379416b24c85862c762abbeede15</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H47" t="n">
+        <v>300</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>5</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L47" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M47" t="n">
+        <v>128</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>30</v>
+      </c>
+      <c r="R47" t="n">
+        <v>100</v>
+      </c>
+      <c r="S47" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T47" t="n">
+        <v>1</v>
+      </c>
+      <c r="U47" t="n">
+        <v>8</v>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-12-04 17:12:29</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/a29b5ed474924a408b848ee089647051</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H48" t="n">
+        <v>300</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>5</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L48" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M48" t="n">
+        <v>128</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>30</v>
+      </c>
+      <c r="R48" t="n">
+        <v>100</v>
+      </c>
+      <c r="S48" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T48" t="n">
+        <v>1</v>
+      </c>
+      <c r="U48" t="n">
+        <v>8</v>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-12-04 17:17:38</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/1c4c0c400d904ed783b05c576bb5bda3</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H49" t="n">
+        <v>300</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>5</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L49" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M49" t="n">
+        <v>128</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>30</v>
+      </c>
+      <c r="R49" t="n">
+        <v>100</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T49" t="n">
+        <v>1</v>
+      </c>
+      <c r="U49" t="n">
+        <v>8</v>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y42"/>
+  <autoFilter ref="A1:Y49"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added SIL and tested on logic circuits
</commit_message>
<xml_diff>
--- a/apps_nicolo/LogicCircuits_4s_5r_MAK_REINFORCE/LogicCircuits_5s_10r_MAK_REINFORCE.xlsx
+++ b/apps_nicolo/LogicCircuits_4s_5r_MAK_REINFORCE/LogicCircuits_5s_10r_MAK_REINFORCE.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$Y$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$Z$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y49"/>
+  <dimension ref="A1:Z72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
@@ -491,6 +491,7 @@
     <col width="80" bestFit="1" customWidth="1" style="7" min="23" max="23"/>
     <col width="135" bestFit="1" customWidth="1" style="7" min="24" max="24"/>
     <col width="19" bestFit="1" customWidth="1" style="7" min="25" max="25"/>
+    <col width="26" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
@@ -4754,8 +4755,1927 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-12-05 09:51:44</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/e6a5c63aacca46f9b0c52cdd8de1de77</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H50" t="n">
+        <v>300</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>5</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L50" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M50" t="n">
+        <v>128</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>30</v>
+      </c>
+      <c r="R50" t="n">
+        <v>100</v>
+      </c>
+      <c r="S50" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T50" t="n">
+        <v>1</v>
+      </c>
+      <c r="U50" t="n">
+        <v>8</v>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-12-05 09:53:19</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/d3251ba440f04698bcad7043a7252e9c</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H51" t="n">
+        <v>300</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>5</v>
+      </c>
+      <c r="K51" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L51" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M51" t="n">
+        <v>128</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>30</v>
+      </c>
+      <c r="R51" t="n">
+        <v>100</v>
+      </c>
+      <c r="S51" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T51" t="n">
+        <v>1</v>
+      </c>
+      <c r="U51" t="n">
+        <v>8</v>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-12-05 09:54:07</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/d0e319d546cd4c9a98a584fe5ff074a5</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H52" t="n">
+        <v>300</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>5</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L52" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M52" t="n">
+        <v>128</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P52" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>30</v>
+      </c>
+      <c r="R52" t="n">
+        <v>100</v>
+      </c>
+      <c r="S52" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T52" t="n">
+        <v>1</v>
+      </c>
+      <c r="U52" t="n">
+        <v>8</v>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2025-12-05 09:54:54</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/5e3e43987e3f4e47bf4591178f5d8497</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H53" t="n">
+        <v>300</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>5</v>
+      </c>
+      <c r="K53" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L53" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M53" t="n">
+        <v>128</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P53" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>30</v>
+      </c>
+      <c r="R53" t="n">
+        <v>100</v>
+      </c>
+      <c r="S53" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T53" t="n">
+        <v>1</v>
+      </c>
+      <c r="U53" t="n">
+        <v>8</v>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2025-12-05 09:58:38</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/f711e15b4bf644a19efa76aa29911cc9</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H54" t="n">
+        <v>300</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>5</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L54" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M54" t="n">
+        <v>128</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P54" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>30</v>
+      </c>
+      <c r="R54" t="n">
+        <v>100</v>
+      </c>
+      <c r="S54" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T54" t="n">
+        <v>1</v>
+      </c>
+      <c r="U54" t="n">
+        <v>8</v>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:05:55</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/1df899cfae0b451aa12456291f70d732</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H55" t="n">
+        <v>300</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>5</v>
+      </c>
+      <c r="K55" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L55" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M55" t="n">
+        <v>128</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P55" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>30</v>
+      </c>
+      <c r="R55" t="n">
+        <v>100</v>
+      </c>
+      <c r="S55" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T55" t="n">
+        <v>1</v>
+      </c>
+      <c r="U55" t="n">
+        <v>8</v>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:14:56</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/a23a2a3695ec4e11ac7cb65a44e2d190</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H56" t="n">
+        <v>300</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>5</v>
+      </c>
+      <c r="K56" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L56" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M56" t="n">
+        <v>128</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P56" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>30</v>
+      </c>
+      <c r="R56" t="n">
+        <v>100</v>
+      </c>
+      <c r="S56" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T56" t="n">
+        <v>1</v>
+      </c>
+      <c r="U56" t="n">
+        <v>8</v>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:17:15</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/fd5ba67aae034ca59571a7daafb218de</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H57" t="n">
+        <v>300</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>5</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L57" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M57" t="n">
+        <v>128</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P57" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>30</v>
+      </c>
+      <c r="R57" t="n">
+        <v>100</v>
+      </c>
+      <c r="S57" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T57" t="n">
+        <v>1</v>
+      </c>
+      <c r="U57" t="n">
+        <v>8</v>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:20:41</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/467560a7a5524fbd85bd4327b279e41d</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H58" t="n">
+        <v>300</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>5</v>
+      </c>
+      <c r="K58" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L58" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M58" t="n">
+        <v>128</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P58" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>30</v>
+      </c>
+      <c r="R58" t="n">
+        <v>100</v>
+      </c>
+      <c r="S58" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T58" t="n">
+        <v>1</v>
+      </c>
+      <c r="U58" t="n">
+        <v>8</v>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:29:05</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/c7968ce2f5574fd3a71f706b03beac02</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H59" t="n">
+        <v>300</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>5</v>
+      </c>
+      <c r="K59" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L59" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M59" t="n">
+        <v>128</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P59" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>30</v>
+      </c>
+      <c r="R59" t="n">
+        <v>100</v>
+      </c>
+      <c r="S59" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T59" t="n">
+        <v>1</v>
+      </c>
+      <c r="U59" t="n">
+        <v>8</v>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:31:26</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/bd630568e7014d509f19ac0f6d393f9e</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H60" t="n">
+        <v>300</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>5</v>
+      </c>
+      <c r="K60" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L60" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M60" t="n">
+        <v>128</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P60" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>30</v>
+      </c>
+      <c r="R60" t="n">
+        <v>100</v>
+      </c>
+      <c r="S60" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T60" t="n">
+        <v>1</v>
+      </c>
+      <c r="U60" t="n">
+        <v>8</v>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:34:24</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/8ad3105cde2c4303824385062207ede0</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H61" t="n">
+        <v>300</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>5</v>
+      </c>
+      <c r="K61" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L61" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M61" t="n">
+        <v>128</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P61" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>30</v>
+      </c>
+      <c r="R61" t="n">
+        <v>100</v>
+      </c>
+      <c r="S61" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T61" t="n">
+        <v>1</v>
+      </c>
+      <c r="U61" t="n">
+        <v>8</v>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:44:02</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/17ed73d2030b44068ff7e24307aa4a54</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H62" t="n">
+        <v>300</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>5</v>
+      </c>
+      <c r="K62" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L62" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M62" t="n">
+        <v>128</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P62" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>30</v>
+      </c>
+      <c r="R62" t="n">
+        <v>100</v>
+      </c>
+      <c r="S62" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T62" t="n">
+        <v>1</v>
+      </c>
+      <c r="U62" t="n">
+        <v>8</v>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:46:26</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/d781a00d114a4b7aaf7ba771b6609dc4</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H63" t="n">
+        <v>300</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>5</v>
+      </c>
+      <c r="K63" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L63" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M63" t="n">
+        <v>128</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P63" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>30</v>
+      </c>
+      <c r="R63" t="n">
+        <v>100</v>
+      </c>
+      <c r="S63" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T63" t="n">
+        <v>1</v>
+      </c>
+      <c r="U63" t="n">
+        <v>8</v>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:47:16</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/aea3f030447946f08bb82520002a548e</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H64" t="n">
+        <v>300</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>5</v>
+      </c>
+      <c r="K64" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L64" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M64" t="n">
+        <v>128</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P64" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>30</v>
+      </c>
+      <c r="R64" t="n">
+        <v>100</v>
+      </c>
+      <c r="S64" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T64" t="n">
+        <v>1</v>
+      </c>
+      <c r="U64" t="n">
+        <v>8</v>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:48:38</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/6148d2d01d58453ab31d6cb5f7f9f905</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H65" t="n">
+        <v>300</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>5</v>
+      </c>
+      <c r="K65" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L65" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M65" t="n">
+        <v>128</v>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P65" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>30</v>
+      </c>
+      <c r="R65" t="n">
+        <v>100</v>
+      </c>
+      <c r="S65" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T65" t="n">
+        <v>1</v>
+      </c>
+      <c r="U65" t="n">
+        <v>8</v>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:48:52</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/3111babfb711428fad4487d5351e8a3a</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H66" t="n">
+        <v>300</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>5</v>
+      </c>
+      <c r="K66" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L66" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M66" t="n">
+        <v>128</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P66" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>30</v>
+      </c>
+      <c r="R66" t="n">
+        <v>100</v>
+      </c>
+      <c r="S66" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T66" t="n">
+        <v>1</v>
+      </c>
+      <c r="U66" t="n">
+        <v>8</v>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:49:45</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/b65e2f1cc0414b849cc04f79cd892d96</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H67" t="n">
+        <v>300</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 128)</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>5</v>
+      </c>
+      <c r="K67" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L67" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M67" t="n">
+        <v>128</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P67" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>30</v>
+      </c>
+      <c r="R67" t="n">
+        <v>100</v>
+      </c>
+      <c r="S67" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T67" t="n">
+        <v>1</v>
+      </c>
+      <c r="U67" t="n">
+        <v>8</v>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2025-12-05 10:57:01</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/72f657787df446549e9d0d3ef9f42423</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H68" t="n">
+        <v>300</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>5</v>
+      </c>
+      <c r="K68" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L68" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M68" t="n">
+        <v>128</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.005, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P68" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>30</v>
+      </c>
+      <c r="R68" t="n">
+        <v>100</v>
+      </c>
+      <c r="S68" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T68" t="n">
+        <v>1</v>
+      </c>
+      <c r="U68" t="n">
+        <v>8</v>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2025-12-05 11:07:28</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/93c3ea3d89a842eca55f1fd5760e4d04</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H69" t="n">
+        <v>300</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>5</v>
+      </c>
+      <c r="K69" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L69" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M69" t="n">
+        <v>128</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P69" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>30</v>
+      </c>
+      <c r="R69" t="n">
+        <v>100</v>
+      </c>
+      <c r="S69" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T69" t="n">
+        <v>1</v>
+      </c>
+      <c r="U69" t="n">
+        <v>8</v>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2025-12-05 11:08:39</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/c7f61f26a0ad470cb65133a02df6c3ae</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H70" t="n">
+        <v>300</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>5</v>
+      </c>
+      <c r="K70" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L70" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M70" t="n">
+        <v>128</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P70" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>30</v>
+      </c>
+      <c r="R70" t="n">
+        <v>100</v>
+      </c>
+      <c r="S70" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T70" t="n">
+        <v>1</v>
+      </c>
+      <c r="U70" t="n">
+        <v>8</v>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2025-12-05 11:24:37</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/8e4a2ca802554357a46f29efd06b4ec3</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H71" t="n">
+        <v>300</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>5</v>
+      </c>
+      <c r="K71" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L71" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M71" t="n">
+        <v>128</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P71" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>30</v>
+      </c>
+      <c r="R71" t="n">
+        <v>100</v>
+      </c>
+      <c r="S71" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T71" t="n">
+        <v>1</v>
+      </c>
+      <c r="U71" t="n">
+        <v>8</v>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>{'sil_loss_weight': 1.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2025-12-05 11:24:56</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-5s-10r-mak-reinforce/39b965da175145a1ae59ace889cb6a20</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H72" t="n">
+        <v>300</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>(5, 4, 3, 1280)</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>5</v>
+      </c>
+      <c r="K72" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L72" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M72" t="n">
+        <v>128</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P72" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>30</v>
+      </c>
+      <c r="R72" t="n">
+        <v>100</v>
+      </c>
+      <c r="S72" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T72" t="n">
+        <v>1</v>
+      </c>
+      <c r="U72" t="n">
+        <v>8</v>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.30072507011480887), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>{'sil_loss_weight': 1.0}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y49"/>
+  <autoFilter ref="A1:Z72"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>